<commit_message>
Siliconomics v0.3：CF19 依 Andy 15:09 定案（維持模型路徑）
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GUUkCEdXKBfReuk3kM2GV9
</commit_message>
<xml_diff>
--- a/siliconomics/model/20261027_Siliconomics_v0.3.xlsx
+++ b/siliconomics/model/20261027_Siliconomics_v0.3.xlsx
@@ -1246,7 +1246,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3754" uniqueCount="1949">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3761" uniqueCount="1955">
   <si>
     <r>
       <rPr>
@@ -1256,7 +1256,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Siliconomics v0.3 — AI </t>
+      <t xml:space="preserve">Siliconomics v0.1 — AI </t>
     </r>
     <r>
       <rPr>
@@ -39065,7 +39065,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">；現值 </t>
+      <t xml:space="preserve">；</t>
     </r>
     <r>
       <rPr>
@@ -39122,7 +39122,694 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">，皆 ≤ </t>
+      <t xml:space="preserve">）。數值維持模型路徑（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Broadcom 90</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">75%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、聯發科 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Marvell 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）；賣方路徑（聯發科 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2028 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">51%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Broadcom </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">需降至約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">26%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）列為聯發科高情境證據。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Andy 2026-10-27 15:09</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：「先這樣，我也沒有更好的數字」</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">已定（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">v0.3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">半導體 索引 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">待判斷 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">CF20</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NVIDIA GPU ABF </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">載板份額合計</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ibiden</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">unimicron</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">nanya_pcb </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">模型 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NVIDIA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">份額合計</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NVIDIA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">側 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026–29 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合計 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">99.0–99.6%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Ibiden 70→59.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、欣興 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25→30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、南電 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2→4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、景碩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2→6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">kinsus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（券商：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Rubin GPU 15–20%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）；本版景碩取剩餘 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2→6%</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">景碩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15–20</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">份額表（合計受限）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本庫建 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">載板份額表合計＝</t>
     </r>
     <r>
       <rPr>
@@ -39141,85 +39828,64 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）。數值預設維持模型路徑；賣方路徑（聯發科 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2028 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">約 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">51%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）列為聯發科高情境證據，待 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Andy </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">決定是否改基準</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">v0.3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（份額表）／待定（數值）</t>
+      <t xml:space="preserve">（含三星電機等）：預設依各公司現值、景碩取剩餘；券商 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15–20% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">列為景碩高情境證據。非 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NVIDIA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">側合計 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">88–89.5% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一併列表</t>
     </r>
   </si>
   <si>
@@ -39250,7 +39916,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2026-10-25 </t>
+      <t xml:space="preserve">2026-10-26 </t>
     </r>
     <r>
       <rPr>
@@ -39269,43 +39935,159 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(1)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">CF20</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NVIDIA GPU ABF </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">載板份額合計</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ibiden</t>
+      <t xml:space="preserve">(14)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">CF21</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">網通（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPO </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金額份額合計 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">29</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">lite 25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
     </r>
     <r>
       <rPr>
@@ -39324,7 +40106,45 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">unimicron</t>
+      <t xml:space="preserve">cohr 10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
     </r>
     <r>
       <rPr>
@@ -39343,67 +40163,162 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">nanya_pcb </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">模型 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NVIDIA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">份額合計</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NVIDIA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">側 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026–29 </t>
-    </r>
+      <t xml:space="preserve">innolight 10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">eoptolink 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">fabrinet 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -39421,83 +40336,365 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">99.0–99.6%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Ibiden 70→59.5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、欣興 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25→30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、南電 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2→4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、景碩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2→6</t>
+      <t xml:space="preserve">55</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">75</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">markets/network CPO </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三情境（無份額表）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NVIDIA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Broadcom CPO </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">份額未建模</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">份額表（無加總檢查）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本庫建 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CPO </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">份額表（含 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NVIDIA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Broadcom </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">交換器端；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Fabrinet </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">代工另列不加總），合計＝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100%</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Siliconomics </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">盤點 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-27 (i)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">CF22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">部署</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">部署 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GW</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">GW</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">network</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">delta</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">quanta </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">等（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI IT capex ÷ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GW IT capex</t>
     </r>
     <r>
       <rPr>
@@ -39510,257 +40707,247 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">kinsus</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（券商：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Rubin GPU 15–20%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）；本版景碩取剩餘 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2→6%</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">景碩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15–20</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">份額表（合計受限）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本庫建 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">GPU </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">載板份額表合計＝</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（含三星電機等）：預設依各公司現值、景碩取剩餘；券商 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15–20% </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">列為景碩高情境證據。非 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NVIDIA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">側合計 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">88–89.5% </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">一併列表</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">半導體 索引 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026-10-26 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">待判斷 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(14)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">CF21</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">網通（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CPO</t>
+    <t xml:space="preserve">23.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amkr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">行業變數（兩算法）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本庫設單一部署 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">路徑（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">R4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上線前以 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">network </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">算法為準），各模型改讀</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Interface — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">下游唯一連結點（各公司模型與市場層只讀本頁 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SIF_ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">具名範圍，經 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">tools/export_snapshot.py </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">匯成版本固定快照）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">節＝輸入（純量，含低／高）；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">節＝推導（年度）；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">節＝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Tokenomics </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">鏡像（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SIF_TK_*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，值＝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TK_In</t>
     </r>
     <r>
       <rPr>
@@ -39777,994 +40964,6 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CPO </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">金額份額合計 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2027</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">28</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">29</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">lite 25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">cohr 10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">innolight 10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">eoptolink 5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">fabrinet 5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">合計 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">55</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">75</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">90</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">markets/network CPO </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">三情境（無份額表）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NVIDIA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Broadcom CPO </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">份額未建模</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">份額表（無加總檢查）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本庫建 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CPO </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">份額表（含 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NVIDIA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Broadcom </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">交換器端；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Fabrinet </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">代工另列不加總），合計＝</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100%</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Siliconomics </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">盤點 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026-10-27 (i)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">CF22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">部署</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">部署 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">GW</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">GW</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">network</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">delta</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">quanta </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">等（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AI IT capex ÷ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">每 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">GW IT capex</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">23.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">amkr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">行業變數（兩算法）</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本庫設單一部署 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">GW </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">路徑（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">R4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">上線前以 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">network </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">算法為準），各模型改讀</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Interface — </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">下游唯一連結點（各公司模型與市場層只讀本頁 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SIF_ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">具名範圍，經 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">tools/export_snapshot.py </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">匯成版本固定快照）。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">A </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">節＝輸入（純量，含低／高）；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">B </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">節＝推導（年度）；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">C </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">節＝</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Tokenomics </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">鏡像（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SIF_TK_*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">，值＝</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">TK_In</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -40778,7 +40977,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Siliconomics v0.3</t>
+      <t xml:space="preserve">Siliconomics v0.1</t>
     </r>
     <r>
       <rPr>
@@ -58259,6 +58458,240 @@
       </rPr>
       <t xml:space="preserve">欄「第二來源／說明」以容納公司模型的第二來源欄</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">S13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">數值</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CF19 TPU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">設計服務份額</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">維持模型路徑（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Broadcom 90</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">75%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、聯發科 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Marvell 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026–28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）；賣方路徑列為聯發科高情境證據</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-27 15:09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">先這樣，我也沒有更好的數字</t>
   </si>
   <si>
     <r>
@@ -68387,7 +68820,7 @@
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">COUNTIF(Conflicts!L4:L25,"待*")</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F58" s="0" t="str">
         <f aca="false">IF(C58=0,"OK","WARN")</f>
@@ -68434,7 +68867,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -68747,6 +69180,29 @@
         <v>1929</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="48.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>1940</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>1941</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>1942</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>1943</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>1944</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>1895</v>
       </c>
     </row>
@@ -68771,7 +69227,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>1939</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -68782,7 +69238,7 @@
         <v>1887</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>1940</v>
+        <v>1946</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>1055</v>
@@ -68791,30 +69247,30 @@
         <v>43</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>1941</v>
+        <v>1947</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>1942</v>
+        <v>1948</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>1943</v>
+        <v>1949</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>1944</v>
+        <v>1950</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>1945</v>
+        <v>1951</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>1946</v>
+        <v>1952</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>1947</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>1948</v>
+        <v>1954</v>
       </c>
     </row>
   </sheetData>
@@ -80194,44 +80650,44 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24" t="s">
+    <row r="22" customFormat="false" ht="111.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>1248</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="2" t="s">
         <v>1249</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="3" t="s">
         <v>1250</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="3" t="s">
         <v>1251</v>
       </c>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="2" t="s">
         <v>1252</v>
       </c>
-      <c r="G22" s="25" t="s">
+      <c r="G22" s="2" t="s">
         <v>1253</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="H22" s="2" t="s">
         <v>1254</v>
       </c>
-      <c r="I22" s="25" t="s">
+      <c r="I22" s="2" t="s">
         <v>1255</v>
       </c>
-      <c r="J22" s="24" t="s">
+      <c r="J22" s="3" t="s">
         <v>1256</v>
       </c>
-      <c r="K22" s="24" t="s">
+      <c r="K22" s="3" t="s">
+        <v>1235</v>
+      </c>
+      <c r="L22" s="2" t="s">
         <v>1257</v>
       </c>
-      <c r="L22" s="25" t="s">
-        <v>1171</v>
-      </c>
-      <c r="M22" s="24" t="s">
+      <c r="M22" s="3" t="s">
         <v>1258</v>
       </c>
     </row>

</xml_diff>